<commit_message>
updating scripts and data
</commit_message>
<xml_diff>
--- a/raw_data/data_org.xlsx
+++ b/raw_data/data_org.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/max/Documents/GitHub/LCOH/raw_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3796E6C1-A029-AE48-9EA8-C4003652C705}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6DBB3B0-151D-F642-815C-4045A305CFB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17040" xr2:uid="{D4AFBB04-8069-EC48-B057-8F20E9E733E9}"/>
+    <workbookView xWindow="4080" yWindow="500" windowWidth="30240" windowHeight="16960" xr2:uid="{D4AFBB04-8069-EC48-B057-8F20E9E733E9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="63">
   <si>
     <t>Data</t>
   </si>
@@ -56,9 +56,6 @@
     <t>Root</t>
   </si>
   <si>
-    <t>fuel prices</t>
-  </si>
-  <si>
     <t>Original_Indices</t>
   </si>
   <si>
@@ -153,6 +150,81 @@
   </si>
   <si>
     <t>steel_tech,comp,</t>
+  </si>
+  <si>
+    <t>fuel prices - AEO2025</t>
+  </si>
+  <si>
+    <t>AEO 2025</t>
+  </si>
+  <si>
+    <t>Census division</t>
+  </si>
+  <si>
+    <t>https://www.eia.gov/outlooks/aeo/</t>
+  </si>
+  <si>
+    <t>Source link</t>
+  </si>
+  <si>
+    <t>Fuel prices, specific to industry</t>
+  </si>
+  <si>
+    <t>Steel producer characteristics</t>
+  </si>
+  <si>
+    <t>FINITO</t>
+  </si>
+  <si>
+    <t>Hydrogen producer characteristics</t>
+  </si>
+  <si>
+    <t>Levelized cost of electricity by technology</t>
+  </si>
+  <si>
+    <t>County</t>
+  </si>
+  <si>
+    <t>https://maps.nrel.gov/slope</t>
+  </si>
+  <si>
+    <t>Fuel prices for electricity and gas</t>
+  </si>
+  <si>
+    <t>EIA</t>
+  </si>
+  <si>
+    <t>State</t>
+  </si>
+  <si>
+    <t>https://www.eia.gov/dnav/ng/ng_pri_sum_a_EPG0_PIN_DMcf_a.htm and https://www.eia.gov/electricity/monthly/</t>
+  </si>
+  <si>
+    <t>CCS characteristics</t>
+  </si>
+  <si>
+    <t>Brown et al</t>
+  </si>
+  <si>
+    <t>Reservoir</t>
+  </si>
+  <si>
+    <t>https://www.mdpi.com/1996-1073/17/15/3780</t>
+  </si>
+  <si>
+    <t>H2 storage site characteristics</t>
+  </si>
+  <si>
+    <t>ReEDS</t>
+  </si>
+  <si>
+    <t>ReEDS Balancing area</t>
+  </si>
+  <si>
+    <t>http://nrel.gov/analysis/reeds/</t>
+  </si>
+  <si>
+    <t>Item</t>
   </si>
 </sst>
 </file>
@@ -188,8 +260,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -524,18 +597,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A13CC789-7EAF-7040-A5F2-C24E6704EB1B}">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="54.1640625" customWidth="1"/>
     <col min="7" max="7" width="21.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B1" t="s">
         <v>4</v>
@@ -550,10 +623,10 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" t="s">
         <v>7</v>
-      </c>
-      <c r="G1" t="s">
-        <v>8</v>
       </c>
       <c r="H1" t="s">
         <v>2</v>
@@ -564,19 +637,19 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
         <v>15</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>16</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>17</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>18</v>
-      </c>
-      <c r="F2" t="s">
-        <v>19</v>
       </c>
       <c r="G2" t="str">
         <f>F2</f>
@@ -585,119 +658,225 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>6</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" t="s">
         <v>9</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>10</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
+        <v>29</v>
+      </c>
+      <c r="J3" t="s">
         <v>11</v>
-      </c>
-      <c r="G3" t="s">
-        <v>30</v>
-      </c>
-      <c r="J3" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
         <v>24</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>25</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>26</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>27</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>28</v>
       </c>
-      <c r="G5" t="s">
-        <v>29</v>
-      </c>
       <c r="H5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" t="s">
         <v>32</v>
       </c>
-      <c r="B6" t="s">
-        <v>33</v>
-      </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" t="s">
         <v>37</v>
-      </c>
-      <c r="G6" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" t="s">
         <v>36</v>
-      </c>
-      <c r="D7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" t="s">
-        <v>18</v>
-      </c>
-      <c r="F7" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C9" t="s">
-        <v>13</v>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="C14" t="s">
+        <v>62</v>
+      </c>
+      <c r="D14" t="s">
+        <v>1</v>
+      </c>
+      <c r="E14" t="s">
+        <v>3</v>
+      </c>
+      <c r="F14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="C15" t="s">
+        <v>43</v>
+      </c>
+      <c r="D15" t="s">
+        <v>39</v>
+      </c>
+      <c r="E15" t="s">
+        <v>40</v>
+      </c>
+      <c r="F15" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="C16" t="s">
+        <v>47</v>
+      </c>
+      <c r="D16" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16" t="s">
+        <v>48</v>
+      </c>
+      <c r="F16" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="17" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="C17" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" t="s">
+        <v>51</v>
+      </c>
+      <c r="E17" t="s">
+        <v>52</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="18" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="C18" t="s">
+        <v>54</v>
+      </c>
+      <c r="D18" t="s">
+        <v>55</v>
+      </c>
+      <c r="E18" t="s">
+        <v>56</v>
+      </c>
+      <c r="F18" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="19" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="C19" t="s">
+        <v>58</v>
+      </c>
+      <c r="D19" t="s">
+        <v>59</v>
+      </c>
+      <c r="E19" t="s">
+        <v>60</v>
+      </c>
+      <c r="F19" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="22" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="C22" t="s">
+        <v>44</v>
+      </c>
+      <c r="D22" t="s">
+        <v>45</v>
+      </c>
+      <c r="E22" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="C23" t="s">
+        <v>46</v>
+      </c>
+      <c r="D23" t="s">
+        <v>45</v>
+      </c>
+      <c r="E23" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>